<commit_message>
US-7 T5: keep the published release column named water_temperature while the model field is surface_temperature
</commit_message>
<xml_diff>
--- a/tests/test_ghfdb/fixtures/sample_ghfdb.xlsx
+++ b/tests/test_ghfdb/fixtures/sample_ghfdb.xlsx
@@ -664,7 +664,7 @@
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>water_temperature</t>
+          <t>Surface_temperature</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>description: water_temperature</t>
+          <t>description: Surface_temperature</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>allowed range: water_temperature</t>
+          <t>allowed range: Surface_temperature</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">

</xml_diff>